<commit_message>
Text file and results update
</commit_message>
<xml_diff>
--- a/results/WIZ_OrdinalPatterns_D5_Monthly_Quarterly.xlsx
+++ b/results/WIZ_OrdinalPatterns_D5_Monthly_Quarterly.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UserA1\Documents\GitHub\Seismic_Amplitude_Timeseries_Analysis\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2792FEFD-C302-4B5E-9037-4510369D121D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F2C4936-8C06-460F-86D0-23FBC0E66EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly" sheetId="1" r:id="rId1"/>
@@ -526,6 +526,7 @@
   <cols>
     <col min="2" max="2" width="12.109375" customWidth="1"/>
     <col min="6" max="6" width="11.109375" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
     <col min="16" max="16" width="16.109375" customWidth="1"/>
     <col min="17" max="17" width="14.5546875" customWidth="1"/>
     <col min="18" max="18" width="11.5546875" customWidth="1"/>

</xml_diff>